<commit_message>
feat: Archivo de configuración de form de respuestas
</commit_message>
<xml_diff>
--- a/data/flujo_conversacional.xlsx
+++ b/data/flujo_conversacional.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ndsabogalv\go\src\github.com\JorgeLo1\chatbot-postgrados-ud\plantillas\flujo_conversacional\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ndsabogalv\go\src\github.com\MrPocketMonsters\herramienta-flujos-rasa\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0999CBEA-B6B6-47CE-A959-B9678CA0DB60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F67DA5A-DC22-40B9-B135-37AA9A9C3B42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_introduccion_libro" sheetId="10" r:id="rId1"/>
@@ -483,9 +483,6 @@
     <t>texto_base</t>
   </si>
   <si>
-    <t>variantes_1_3</t>
-  </si>
-  <si>
     <t>fallback_asociado</t>
   </si>
   <si>
@@ -1039,6 +1036,9 @@
   </si>
   <si>
     <t>slot_dependencia_responsable</t>
+  </si>
+  <si>
+    <t>variantes</t>
   </si>
 </sst>
 </file>
@@ -1112,10 +1112,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1344,6 +1344,33 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1379,33 +1406,6 @@
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1420,10 +1420,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{94F28579-0618-4E96-AA7D-A0B2ED44AB9A}" name="Tabla10" displayName="Tabla10" ref="A1:A4" totalsRowShown="0" headerRowDxfId="79" dataDxfId="78">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{94F28579-0618-4E96-AA7D-A0B2ED44AB9A}" name="Tabla10" displayName="Tabla10" ref="A1:A4" totalsRowShown="0" headerRowDxfId="88" dataDxfId="87">
   <autoFilter ref="A1:A4" xr:uid="{94F28579-0618-4E96-AA7D-A0B2ED44AB9A}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{69C95A58-1AA1-42C9-9B8D-2D2310442EFD}" name="introduccion" dataDxfId="77"/>
+    <tableColumn id="1" xr3:uid="{69C95A58-1AA1-42C9-9B8D-2D2310442EFD}" name="introduccion" dataDxfId="86"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1443,16 +1443,16 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B6ECAECC-7F11-473F-A3F8-9434400EAF6D}" name="Tabla1" displayName="Tabla1" ref="A2:G23" totalsRowShown="0" headerRowDxfId="88" dataDxfId="87">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B6ECAECC-7F11-473F-A3F8-9434400EAF6D}" name="Tabla1" displayName="Tabla1" ref="A2:G23" totalsRowShown="0" headerRowDxfId="85" dataDxfId="84">
   <autoFilter ref="A2:G23" xr:uid="{B6ECAECC-7F11-473F-A3F8-9434400EAF6D}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{C6EE0453-DD5E-455E-8F32-1728324AD9E8}" name="flujo_id" dataDxfId="86"/>
-    <tableColumn id="2" xr3:uid="{30F056C8-5C87-4FF2-858F-D1E3DF8CA1DA}" name="objetivo" dataDxfId="85"/>
-    <tableColumn id="3" xr3:uid="{2271D532-BFD3-4A68-A7D3-B86D4BC7D1ED}" name="alcance" dataDxfId="84"/>
-    <tableColumn id="4" xr3:uid="{795E787F-72E2-4193-84DB-AF0D60DDAA1C}" name="in_scope" dataDxfId="83"/>
-    <tableColumn id="5" xr3:uid="{680BF66C-7F03-4798-8067-26134579085C}" name="out_scope" dataDxfId="82"/>
-    <tableColumn id="6" xr3:uid="{0DF659C7-BB96-4FDA-9B29-2F9F7ABFD7ED}" name="criterio_cierre" dataDxfId="81"/>
-    <tableColumn id="7" xr3:uid="{BF120C84-0B4B-43C8-A237-98E660EF0C4A}" name="criterio_cierre_operativo" dataDxfId="80"/>
+    <tableColumn id="1" xr3:uid="{C6EE0453-DD5E-455E-8F32-1728324AD9E8}" name="flujo_id" dataDxfId="83"/>
+    <tableColumn id="2" xr3:uid="{30F056C8-5C87-4FF2-858F-D1E3DF8CA1DA}" name="objetivo" dataDxfId="82"/>
+    <tableColumn id="3" xr3:uid="{2271D532-BFD3-4A68-A7D3-B86D4BC7D1ED}" name="alcance" dataDxfId="81"/>
+    <tableColumn id="4" xr3:uid="{795E787F-72E2-4193-84DB-AF0D60DDAA1C}" name="in_scope" dataDxfId="80"/>
+    <tableColumn id="5" xr3:uid="{680BF66C-7F03-4798-8067-26134579085C}" name="out_scope" dataDxfId="79"/>
+    <tableColumn id="6" xr3:uid="{0DF659C7-BB96-4FDA-9B29-2F9F7ABFD7ED}" name="criterio_cierre" dataDxfId="78"/>
+    <tableColumn id="7" xr3:uid="{BF120C84-0B4B-43C8-A237-98E660EF0C4A}" name="criterio_cierre_operativo" dataDxfId="77"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1526,7 +1526,7 @@
     <tableColumn id="5" xr3:uid="{A4ED9A37-33FB-48DE-9396-DDFEAC9D5099}" name="longitud" dataDxfId="34"/>
     <tableColumn id="6" xr3:uid="{7173C801-3241-4CFE-831D-B2605A556AB3}" name="contenido_obligatorio" dataDxfId="33"/>
     <tableColumn id="7" xr3:uid="{091B581B-865B-4BA8-BE97-1484592C7898}" name="texto_base" dataDxfId="32"/>
-    <tableColumn id="8" xr3:uid="{AB483609-B2F9-4FFC-8A32-88355DE63F46}" name="variantes_1_3" dataDxfId="31"/>
+    <tableColumn id="8" xr3:uid="{AB483609-B2F9-4FFC-8A32-88355DE63F46}" name="variantes" dataDxfId="31"/>
     <tableColumn id="9" xr3:uid="{2638628A-D494-4933-8397-FC91F4C31DF6}" name="fallback_asociado" dataDxfId="30"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1850,22 +1850,22 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
   </sheetData>
@@ -1889,39 +1889,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
-        <v>311</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
+      <c r="A1" s="9" t="s">
+        <v>310</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
     </row>
     <row r="2" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>16</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>236</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>312</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>313</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>314</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -1929,10 +1929,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>238</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -1940,10 +1940,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -1951,10 +1951,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -1962,10 +1962,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -1973,10 +1973,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -1984,10 +1984,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -1995,10 +1995,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -2006,10 +2006,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -2017,10 +2017,10 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -2028,10 +2028,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -2054,15 +2054,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
+      <c r="A1" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
     </row>
     <row r="2" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -2089,25 +2089,25 @@
     </row>
     <row r="3" spans="1:7" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="C3" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="D3" s="5" t="s">
         <v>255</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="E3" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>258</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="45" x14ac:dyDescent="0.25">
@@ -2158,18 +2158,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
-        <v>260</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
+      <c r="A1" s="9" t="s">
+        <v>259</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -2205,34 +2205,34 @@
     </row>
     <row r="3" spans="1:10" s="7" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="C3" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>263</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>265</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="H3" s="6" t="s">
         <v>267</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="I3" s="6" t="s">
         <v>268</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="J3" s="6" t="s">
         <v>269</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2441,18 +2441,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
-        <v>272</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
+      <c r="A1" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -2488,34 +2488,34 @@
     </row>
     <row r="3" spans="1:10" s="7" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>274</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>275</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>276</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="H3" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="I3" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="J3" s="6" t="s">
         <v>280</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -2733,18 +2733,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
-        <v>326</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
+      <c r="A1" s="9" t="s">
+        <v>325</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -2780,34 +2780,34 @@
     </row>
     <row r="3" spans="1:10" s="7" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>327</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>282</v>
-      </c>
-      <c r="D3" s="5" t="s">
+      <c r="F3" s="8" t="s">
         <v>283</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>328</v>
-      </c>
-      <c r="F3" s="9" t="s">
+      <c r="G3" s="8" t="s">
         <v>284</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="H3" s="5" t="s">
         <v>285</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>286</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="J3" s="5" t="s">
         <v>287</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -2824,7 +2824,7 @@
         <v>27</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>118</v>
@@ -2856,7 +2856,7 @@
         <v>33</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>118</v>
@@ -2888,7 +2888,7 @@
         <v>33</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>128</v>
@@ -2920,7 +2920,7 @@
         <v>40</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>128</v>
@@ -2952,7 +2952,7 @@
         <v>46</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>118</v>
@@ -2984,7 +2984,7 @@
         <v>40</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>118</v>
@@ -3025,17 +3025,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
-        <v>289</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
+      <c r="A1" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
     </row>
     <row r="2" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -3060,39 +3060,39 @@
         <v>148</v>
       </c>
       <c r="H2" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:9" s="7" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>291</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="H3" s="6" t="s">
         <v>295</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="I3" s="6" t="s">
         <v>296</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>297</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="75" x14ac:dyDescent="0.25">
@@ -3106,22 +3106,22 @@
         <v>23</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="75" x14ac:dyDescent="0.25">
@@ -3135,22 +3135,22 @@
         <v>27</v>
       </c>
       <c r="D5" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="H5" s="2" t="s">
-        <v>160</v>
-      </c>
       <c r="I5" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="60" x14ac:dyDescent="0.25">
@@ -3164,22 +3164,22 @@
         <v>33</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E6" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="H6" s="2" t="s">
-        <v>164</v>
-      </c>
       <c r="I6" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
@@ -3193,22 +3193,22 @@
         <v>40</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F7" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="H7" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="H7" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="I7" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="75" x14ac:dyDescent="0.25">
@@ -3222,22 +3222,22 @@
         <v>46</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F8" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="H8" s="2" t="s">
-        <v>170</v>
-      </c>
       <c r="I8" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="75" x14ac:dyDescent="0.25">
@@ -3251,22 +3251,22 @@
         <v>52</v>
       </c>
       <c r="D9" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>152</v>
-      </c>
       <c r="F9" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>173</v>
-      </c>
       <c r="I9" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -3290,53 +3290,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
-        <v>317</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
+      <c r="A1" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
     </row>
     <row r="2" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>177</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:6" s="7" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>315</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>298</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>318</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>316</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>319</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -3344,10 +3344,10 @@
         <v>7</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>179</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>180</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>69</v>
@@ -3356,7 +3356,7 @@
         <v>28</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -3364,10 +3364,10 @@
         <v>7</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>182</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>183</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>76</v>
@@ -3376,7 +3376,7 @@
         <v>41</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -3384,10 +3384,10 @@
         <v>7</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>185</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>186</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>83</v>
@@ -3396,7 +3396,7 @@
         <v>47</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -3404,10 +3404,10 @@
         <v>7</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>188</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>189</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>89</v>
@@ -3416,7 +3416,7 @@
         <v>53</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -3424,10 +3424,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>101</v>
@@ -3436,7 +3436,7 @@
         <v>59</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="45" x14ac:dyDescent="0.25">
@@ -3444,19 +3444,19 @@
         <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>321</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>322</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>324</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -3481,39 +3481,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
-        <v>320</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
+      <c r="A1" s="9" t="s">
+        <v>319</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
     </row>
     <row r="2" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>194</v>
-      </c>
       <c r="D2" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="7" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>300</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>302</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="165" x14ac:dyDescent="0.25">
@@ -3521,13 +3521,13 @@
         <v>7</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>196</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="60" x14ac:dyDescent="0.25">
@@ -3535,13 +3535,13 @@
         <v>7</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>199</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -3565,67 +3565,67 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
-        <v>303</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
+      <c r="A1" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>206</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="3" spans="1:8" s="7" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>304</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>305</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>306</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>307</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="H3" s="6" t="s">
         <v>309</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="45" x14ac:dyDescent="0.25">
@@ -3633,25 +3633,25 @@
         <v>7</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>213</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -3659,25 +3659,25 @@
         <v>7</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>220</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="45" x14ac:dyDescent="0.25">
@@ -3685,25 +3685,25 @@
         <v>7</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>227</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="45" x14ac:dyDescent="0.25">
@@ -3711,25 +3711,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>230</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>231</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>135</v>
       </c>
       <c r="F7" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="H7" s="2" t="s">
         <v>233</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>